<commit_message>
chore: refresh the time-course report from the CI artefact
</commit_message>
<xml_diff>
--- a/examples/TimeCourse_Niepel_CellSyst_2019/report/v1/raw_data/MN20160421_X04 total.xlsx
+++ b/examples/TimeCourse_Niepel_CellSyst_2019/report/v1/raw_data/MN20160421_X04 total.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6519" uniqueCount="5342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6209" uniqueCount="5116">
   <si>
     <t>Label: MN20160421_X04</t>
   </si>
@@ -15362,684 +15362,6 @@
   </si>
   <si>
     <t>6745</t>
-  </si>
-  <si>
-    <t>4/25/2016 5:05:00 PM</t>
-  </si>
-  <si>
-    <t>76</t>
-  </si>
-  <si>
-    <t>3385</t>
-  </si>
-  <si>
-    <t>11361</t>
-  </si>
-  <si>
-    <t>12145</t>
-  </si>
-  <si>
-    <t>14059</t>
-  </si>
-  <si>
-    <t>8198</t>
-  </si>
-  <si>
-    <t>9869</t>
-  </si>
-  <si>
-    <t>10771</t>
-  </si>
-  <si>
-    <t>9721</t>
-  </si>
-  <si>
-    <t>15653</t>
-  </si>
-  <si>
-    <t>16355</t>
-  </si>
-  <si>
-    <t>6901</t>
-  </si>
-  <si>
-    <t>17046</t>
-  </si>
-  <si>
-    <t>6735</t>
-  </si>
-  <si>
-    <t>19479</t>
-  </si>
-  <si>
-    <t>9295</t>
-  </si>
-  <si>
-    <t>2697</t>
-  </si>
-  <si>
-    <t>5345</t>
-  </si>
-  <si>
-    <t>16376</t>
-  </si>
-  <si>
-    <t>6889</t>
-  </si>
-  <si>
-    <t>5468</t>
-  </si>
-  <si>
-    <t>16154</t>
-  </si>
-  <si>
-    <t>16588</t>
-  </si>
-  <si>
-    <t>18844</t>
-  </si>
-  <si>
-    <t>5143</t>
-  </si>
-  <si>
-    <t>6854</t>
-  </si>
-  <si>
-    <t>19284</t>
-  </si>
-  <si>
-    <t>15892</t>
-  </si>
-  <si>
-    <t>6490</t>
-  </si>
-  <si>
-    <t>15721</t>
-  </si>
-  <si>
-    <t>15392</t>
-  </si>
-  <si>
-    <t>5277</t>
-  </si>
-  <si>
-    <t>18449</t>
-  </si>
-  <si>
-    <t>14962</t>
-  </si>
-  <si>
-    <t>9703</t>
-  </si>
-  <si>
-    <t>18559</t>
-  </si>
-  <si>
-    <t>5361</t>
-  </si>
-  <si>
-    <t>19819</t>
-  </si>
-  <si>
-    <t>16774</t>
-  </si>
-  <si>
-    <t>3365</t>
-  </si>
-  <si>
-    <t>16138</t>
-  </si>
-  <si>
-    <t>18492</t>
-  </si>
-  <si>
-    <t>5706</t>
-  </si>
-  <si>
-    <t>17714</t>
-  </si>
-  <si>
-    <t>18735</t>
-  </si>
-  <si>
-    <t>18425</t>
-  </si>
-  <si>
-    <t>13338</t>
-  </si>
-  <si>
-    <t>2904</t>
-  </si>
-  <si>
-    <t>6938</t>
-  </si>
-  <si>
-    <t>14082</t>
-  </si>
-  <si>
-    <t>18907</t>
-  </si>
-  <si>
-    <t>10902</t>
-  </si>
-  <si>
-    <t>8130</t>
-  </si>
-  <si>
-    <t>18652</t>
-  </si>
-  <si>
-    <t>19239</t>
-  </si>
-  <si>
-    <t>11260</t>
-  </si>
-  <si>
-    <t>4878</t>
-  </si>
-  <si>
-    <t>5332</t>
-  </si>
-  <si>
-    <t>11946</t>
-  </si>
-  <si>
-    <t>20045</t>
-  </si>
-  <si>
-    <t>17141</t>
-  </si>
-  <si>
-    <t>5405</t>
-  </si>
-  <si>
-    <t>9187</t>
-  </si>
-  <si>
-    <t>19406</t>
-  </si>
-  <si>
-    <t>19516</t>
-  </si>
-  <si>
-    <t>19789</t>
-  </si>
-  <si>
-    <t>21245</t>
-  </si>
-  <si>
-    <t>18745</t>
-  </si>
-  <si>
-    <t>13200</t>
-  </si>
-  <si>
-    <t>18854</t>
-  </si>
-  <si>
-    <t>19522</t>
-  </si>
-  <si>
-    <t>18791</t>
-  </si>
-  <si>
-    <t>19104</t>
-  </si>
-  <si>
-    <t>7804</t>
-  </si>
-  <si>
-    <t>8254</t>
-  </si>
-  <si>
-    <t>19476</t>
-  </si>
-  <si>
-    <t>18691</t>
-  </si>
-  <si>
-    <t>14517</t>
-  </si>
-  <si>
-    <t>3723</t>
-  </si>
-  <si>
-    <t>17057</t>
-  </si>
-  <si>
-    <t>18825</t>
-  </si>
-  <si>
-    <t>8558</t>
-  </si>
-  <si>
-    <t>14721</t>
-  </si>
-  <si>
-    <t>19562</t>
-  </si>
-  <si>
-    <t>8402</t>
-  </si>
-  <si>
-    <t>15575</t>
-  </si>
-  <si>
-    <t>19432</t>
-  </si>
-  <si>
-    <t>14812</t>
-  </si>
-  <si>
-    <t>19764</t>
-  </si>
-  <si>
-    <t>18795</t>
-  </si>
-  <si>
-    <t>19995</t>
-  </si>
-  <si>
-    <t>19257</t>
-  </si>
-  <si>
-    <t>19199</t>
-  </si>
-  <si>
-    <t>16799</t>
-  </si>
-  <si>
-    <t>11968</t>
-  </si>
-  <si>
-    <t>19818</t>
-  </si>
-  <si>
-    <t>8861</t>
-  </si>
-  <si>
-    <t>20707</t>
-  </si>
-  <si>
-    <t>10814</t>
-  </si>
-  <si>
-    <t>2848</t>
-  </si>
-  <si>
-    <t>18983</t>
-  </si>
-  <si>
-    <t>18405</t>
-  </si>
-  <si>
-    <t>17838</t>
-  </si>
-  <si>
-    <t>18173</t>
-  </si>
-  <si>
-    <t>19070</t>
-  </si>
-  <si>
-    <t>10263</t>
-  </si>
-  <si>
-    <t>8217</t>
-  </si>
-  <si>
-    <t>20366</t>
-  </si>
-  <si>
-    <t>17746</t>
-  </si>
-  <si>
-    <t>13582</t>
-  </si>
-  <si>
-    <t>7801</t>
-  </si>
-  <si>
-    <t>5923</t>
-  </si>
-  <si>
-    <t>8678</t>
-  </si>
-  <si>
-    <t>18602</t>
-  </si>
-  <si>
-    <t>12664</t>
-  </si>
-  <si>
-    <t>20416</t>
-  </si>
-  <si>
-    <t>11859</t>
-  </si>
-  <si>
-    <t>20013</t>
-  </si>
-  <si>
-    <t>19952</t>
-  </si>
-  <si>
-    <t>7944</t>
-  </si>
-  <si>
-    <t>6990</t>
-  </si>
-  <si>
-    <t>5905</t>
-  </si>
-  <si>
-    <t>13371</t>
-  </si>
-  <si>
-    <t>19765</t>
-  </si>
-  <si>
-    <t>17358</t>
-  </si>
-  <si>
-    <t>6940</t>
-  </si>
-  <si>
-    <t>12829</t>
-  </si>
-  <si>
-    <t>19356</t>
-  </si>
-  <si>
-    <t>19174</t>
-  </si>
-  <si>
-    <t>8241</t>
-  </si>
-  <si>
-    <t>21083</t>
-  </si>
-  <si>
-    <t>9525</t>
-  </si>
-  <si>
-    <t>7642</t>
-  </si>
-  <si>
-    <t>19628</t>
-  </si>
-  <si>
-    <t>18846</t>
-  </si>
-  <si>
-    <t>18232</t>
-  </si>
-  <si>
-    <t>8357</t>
-  </si>
-  <si>
-    <t>19762</t>
-  </si>
-  <si>
-    <t>3458</t>
-  </si>
-  <si>
-    <t>20182</t>
-  </si>
-  <si>
-    <t>4894</t>
-  </si>
-  <si>
-    <t>11904</t>
-  </si>
-  <si>
-    <t>17414</t>
-  </si>
-  <si>
-    <t>18537</t>
-  </si>
-  <si>
-    <t>11374</t>
-  </si>
-  <si>
-    <t>7332</t>
-  </si>
-  <si>
-    <t>16299</t>
-  </si>
-  <si>
-    <t>19306</t>
-  </si>
-  <si>
-    <t>19086</t>
-  </si>
-  <si>
-    <t>13467</t>
-  </si>
-  <si>
-    <t>20209</t>
-  </si>
-  <si>
-    <t>4563</t>
-  </si>
-  <si>
-    <t>14780</t>
-  </si>
-  <si>
-    <t>19184</t>
-  </si>
-  <si>
-    <t>19313</t>
-  </si>
-  <si>
-    <t>19878</t>
-  </si>
-  <si>
-    <t>18429</t>
-  </si>
-  <si>
-    <t>18722</t>
-  </si>
-  <si>
-    <t>19318</t>
-  </si>
-  <si>
-    <t>19532</t>
-  </si>
-  <si>
-    <t>11960</t>
-  </si>
-  <si>
-    <t>12863</t>
-  </si>
-  <si>
-    <t>13554</t>
-  </si>
-  <si>
-    <t>8508</t>
-  </si>
-  <si>
-    <t>6803</t>
-  </si>
-  <si>
-    <t>8409</t>
-  </si>
-  <si>
-    <t>4835</t>
-  </si>
-  <si>
-    <t>19219</t>
-  </si>
-  <si>
-    <t>18815</t>
-  </si>
-  <si>
-    <t>6010</t>
-  </si>
-  <si>
-    <t>17608</t>
-  </si>
-  <si>
-    <t>20164</t>
-  </si>
-  <si>
-    <t>19252</t>
-  </si>
-  <si>
-    <t>2934</t>
-  </si>
-  <si>
-    <t>6597</t>
-  </si>
-  <si>
-    <t>14927</t>
-  </si>
-  <si>
-    <t>18969</t>
-  </si>
-  <si>
-    <t>18228</t>
-  </si>
-  <si>
-    <t>16278</t>
-  </si>
-  <si>
-    <t>18922</t>
-  </si>
-  <si>
-    <t>5442</t>
-  </si>
-  <si>
-    <t>20192</t>
-  </si>
-  <si>
-    <t>6454</t>
-  </si>
-  <si>
-    <t>17725</t>
-  </si>
-  <si>
-    <t>3462</t>
-  </si>
-  <si>
-    <t>11039</t>
-  </si>
-  <si>
-    <t>13952</t>
-  </si>
-  <si>
-    <t>18386</t>
-  </si>
-  <si>
-    <t>18845</t>
-  </si>
-  <si>
-    <t>2918</t>
-  </si>
-  <si>
-    <t>2913</t>
-  </si>
-  <si>
-    <t>20286</t>
-  </si>
-  <si>
-    <t>18999</t>
-  </si>
-  <si>
-    <t>10783</t>
-  </si>
-  <si>
-    <t>14867</t>
-  </si>
-  <si>
-    <t>2800</t>
-  </si>
-  <si>
-    <t>16240</t>
-  </si>
-  <si>
-    <t>13060</t>
-  </si>
-  <si>
-    <t>14908</t>
-  </si>
-  <si>
-    <t>19639</t>
-  </si>
-  <si>
-    <t>13846</t>
-  </si>
-  <si>
-    <t>19966</t>
-  </si>
-  <si>
-    <t>20133</t>
-  </si>
-  <si>
-    <t>20716</t>
-  </si>
-  <si>
-    <t>16684</t>
-  </si>
-  <si>
-    <t>3449</t>
-  </si>
-  <si>
-    <t>16967</t>
-  </si>
-  <si>
-    <t>19367</t>
-  </si>
-  <si>
-    <t>19641</t>
-  </si>
-  <si>
-    <t>14336</t>
-  </si>
-  <si>
-    <t>2896</t>
-  </si>
-  <si>
-    <t>16245</t>
-  </si>
-  <si>
-    <t>20326</t>
-  </si>
-  <si>
-    <t>13950</t>
-  </si>
-  <si>
-    <t>17568</t>
-  </si>
-  <si>
-    <t>17855</t>
-  </si>
-  <si>
-    <t>11214</t>
-  </si>
-  <si>
-    <t>11956</t>
-  </si>
-  <si>
-    <t>18696</t>
-  </si>
-  <si>
-    <t>19910</t>
-  </si>
-  <si>
-    <t>6831</t>
-  </si>
-  <si>
-    <t>18732</t>
-  </si>
-  <si>
-    <t>13695</t>
-  </si>
-  <si>
-    <t>6649</t>
-  </si>
-  <si>
-    <t>11019</t>
   </si>
 </sst>
 </file>
@@ -16371,7 +15693,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:KX30"/>
+  <dimension ref="A1:KX29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:310">
@@ -35057,938 +34379,6 @@
         <v>2939</v>
       </c>
     </row>
-    <row r="30" spans="1:310">
-      <c r="A30" t="s">
-        <v>5116</v>
-      </c>
-      <c r="B30" t="s">
-        <v>5117</v>
-      </c>
-      <c r="C30" t="s">
-        <v>5118</v>
-      </c>
-      <c r="D30" t="s">
-        <v>934</v>
-      </c>
-      <c r="E30" t="s">
-        <v>5119</v>
-      </c>
-      <c r="F30" t="s">
-        <v>5120</v>
-      </c>
-      <c r="G30" t="s">
-        <v>5121</v>
-      </c>
-      <c r="H30" t="s">
-        <v>5122</v>
-      </c>
-      <c r="I30" t="s">
-        <v>5123</v>
-      </c>
-      <c r="J30" t="s">
-        <v>5124</v>
-      </c>
-      <c r="K30" t="s">
-        <v>1605</v>
-      </c>
-      <c r="L30" t="s">
-        <v>5125</v>
-      </c>
-      <c r="M30" t="s">
-        <v>5126</v>
-      </c>
-      <c r="N30" t="s">
-        <v>4629</v>
-      </c>
-      <c r="O30" t="s">
-        <v>5127</v>
-      </c>
-      <c r="P30" t="s">
-        <v>742</v>
-      </c>
-      <c r="Q30" t="s">
-        <v>5128</v>
-      </c>
-      <c r="R30" t="s">
-        <v>5129</v>
-      </c>
-      <c r="S30" t="s">
-        <v>1795</v>
-      </c>
-      <c r="T30" t="s">
-        <v>679</v>
-      </c>
-      <c r="U30" t="s">
-        <v>4649</v>
-      </c>
-      <c r="V30" t="s">
-        <v>5130</v>
-      </c>
-      <c r="W30" t="s">
-        <v>5131</v>
-      </c>
-      <c r="X30" t="s">
-        <v>2367</v>
-      </c>
-      <c r="Y30" t="s">
-        <v>5132</v>
-      </c>
-      <c r="Z30" t="s">
-        <v>4298</v>
-      </c>
-      <c r="AA30" t="s">
-        <v>1383</v>
-      </c>
-      <c r="AB30" t="s">
-        <v>5133</v>
-      </c>
-      <c r="AC30" t="s">
-        <v>5134</v>
-      </c>
-      <c r="AD30" t="s">
-        <v>5135</v>
-      </c>
-      <c r="AE30" t="s">
-        <v>3447</v>
-      </c>
-      <c r="AF30" t="s">
-        <v>1583</v>
-      </c>
-      <c r="AG30" t="s">
-        <v>5136</v>
-      </c>
-      <c r="AH30" t="s">
-        <v>5137</v>
-      </c>
-      <c r="AI30" t="s">
-        <v>5138</v>
-      </c>
-      <c r="AJ30" t="s">
-        <v>1101</v>
-      </c>
-      <c r="AK30" t="s">
-        <v>5139</v>
-      </c>
-      <c r="AL30" t="s">
-        <v>5140</v>
-      </c>
-      <c r="AM30" t="s">
-        <v>5141</v>
-      </c>
-      <c r="AN30" t="s">
-        <v>5142</v>
-      </c>
-      <c r="AO30" t="s">
-        <v>5143</v>
-      </c>
-      <c r="AP30" t="s">
-        <v>4498</v>
-      </c>
-      <c r="AQ30" t="s">
-        <v>5144</v>
-      </c>
-      <c r="AR30" t="s">
-        <v>5145</v>
-      </c>
-      <c r="AS30" t="s">
-        <v>1069</v>
-      </c>
-      <c r="AT30" t="s">
-        <v>5146</v>
-      </c>
-      <c r="AU30" t="s">
-        <v>1638</v>
-      </c>
-      <c r="AV30" t="s">
-        <v>5147</v>
-      </c>
-      <c r="AW30" t="s">
-        <v>5148</v>
-      </c>
-      <c r="AX30" t="s">
-        <v>408</v>
-      </c>
-      <c r="AY30" t="s">
-        <v>5149</v>
-      </c>
-      <c r="AZ30" t="s">
-        <v>5150</v>
-      </c>
-      <c r="BA30" t="s">
-        <v>2025</v>
-      </c>
-      <c r="BB30" t="s">
-        <v>5151</v>
-      </c>
-      <c r="BC30" t="s">
-        <v>5152</v>
-      </c>
-      <c r="BD30" t="s">
-        <v>5153</v>
-      </c>
-      <c r="BE30" t="s">
-        <v>5154</v>
-      </c>
-      <c r="BF30" t="s">
-        <v>5155</v>
-      </c>
-      <c r="BG30" t="s">
-        <v>2320</v>
-      </c>
-      <c r="BH30" t="s">
-        <v>5156</v>
-      </c>
-      <c r="BI30" t="s">
-        <v>5157</v>
-      </c>
-      <c r="BJ30" t="s">
-        <v>5158</v>
-      </c>
-      <c r="BK30" t="s">
-        <v>5159</v>
-      </c>
-      <c r="BL30" t="s">
-        <v>5160</v>
-      </c>
-      <c r="BM30" t="s">
-        <v>5161</v>
-      </c>
-      <c r="BN30" t="s">
-        <v>5162</v>
-      </c>
-      <c r="BO30" t="s">
-        <v>3748</v>
-      </c>
-      <c r="BP30" t="s">
-        <v>5163</v>
-      </c>
-      <c r="BQ30" t="s">
-        <v>5164</v>
-      </c>
-      <c r="BR30" t="s">
-        <v>3635</v>
-      </c>
-      <c r="BS30" t="s">
-        <v>4071</v>
-      </c>
-      <c r="BT30" t="s">
-        <v>3894</v>
-      </c>
-      <c r="BU30" t="s">
-        <v>5165</v>
-      </c>
-      <c r="BV30" t="s">
-        <v>5166</v>
-      </c>
-      <c r="BW30" t="s">
-        <v>5167</v>
-      </c>
-      <c r="BX30" t="s">
-        <v>3806</v>
-      </c>
-      <c r="BY30" t="s">
-        <v>5168</v>
-      </c>
-      <c r="BZ30" t="s">
-        <v>5169</v>
-      </c>
-      <c r="CA30" t="s">
-        <v>4396</v>
-      </c>
-      <c r="CB30" t="s">
-        <v>5170</v>
-      </c>
-      <c r="CC30" t="s">
-        <v>4016</v>
-      </c>
-      <c r="CD30" t="s">
-        <v>4498</v>
-      </c>
-      <c r="CE30" t="s">
-        <v>2778</v>
-      </c>
-      <c r="CF30" t="s">
-        <v>5171</v>
-      </c>
-      <c r="CG30" t="s">
-        <v>5172</v>
-      </c>
-      <c r="CH30" t="s">
-        <v>5173</v>
-      </c>
-      <c r="CI30" t="s">
-        <v>2915</v>
-      </c>
-      <c r="CJ30" t="s">
-        <v>5174</v>
-      </c>
-      <c r="CK30" t="s">
-        <v>4423</v>
-      </c>
-      <c r="CL30" t="s">
-        <v>5175</v>
-      </c>
-      <c r="CM30" t="s">
-        <v>5176</v>
-      </c>
-      <c r="CN30" t="s">
-        <v>5177</v>
-      </c>
-      <c r="CO30" t="s">
-        <v>5178</v>
-      </c>
-      <c r="CP30" t="s">
-        <v>5179</v>
-      </c>
-      <c r="CQ30" t="s">
-        <v>5180</v>
-      </c>
-      <c r="CR30" t="s">
-        <v>2154</v>
-      </c>
-      <c r="CS30" t="s">
-        <v>5181</v>
-      </c>
-      <c r="CT30" t="s">
-        <v>5182</v>
-      </c>
-      <c r="CU30" t="s">
-        <v>5183</v>
-      </c>
-      <c r="CV30" t="s">
-        <v>5184</v>
-      </c>
-      <c r="CW30" t="s">
-        <v>5185</v>
-      </c>
-      <c r="CX30" t="s">
-        <v>5186</v>
-      </c>
-      <c r="CY30" t="s">
-        <v>5187</v>
-      </c>
-      <c r="CZ30" t="s">
-        <v>5188</v>
-      </c>
-      <c r="DA30" t="s">
-        <v>5189</v>
-      </c>
-      <c r="DB30" t="s">
-        <v>5190</v>
-      </c>
-      <c r="DC30" t="s">
-        <v>1027</v>
-      </c>
-      <c r="DD30" t="s">
-        <v>5191</v>
-      </c>
-      <c r="DE30" t="s">
-        <v>5192</v>
-      </c>
-      <c r="DF30" t="s">
-        <v>5193</v>
-      </c>
-      <c r="DG30" t="s">
-        <v>5194</v>
-      </c>
-      <c r="DH30" t="s">
-        <v>3262</v>
-      </c>
-      <c r="DI30" t="s">
-        <v>5195</v>
-      </c>
-      <c r="DJ30" t="s">
-        <v>1164</v>
-      </c>
-      <c r="DK30" t="s">
-        <v>5196</v>
-      </c>
-      <c r="DL30" t="s">
-        <v>5197</v>
-      </c>
-      <c r="DM30" t="s">
-        <v>5198</v>
-      </c>
-      <c r="DN30" t="s">
-        <v>4468</v>
-      </c>
-      <c r="DO30" t="s">
-        <v>3855</v>
-      </c>
-      <c r="DP30" t="s">
-        <v>5199</v>
-      </c>
-      <c r="DQ30" t="s">
-        <v>5200</v>
-      </c>
-      <c r="DR30" t="s">
-        <v>5201</v>
-      </c>
-      <c r="DS30" t="s">
-        <v>5202</v>
-      </c>
-      <c r="DT30" t="s">
-        <v>5083</v>
-      </c>
-      <c r="DU30" t="s">
-        <v>5203</v>
-      </c>
-      <c r="DV30" t="s">
-        <v>5204</v>
-      </c>
-      <c r="DW30" t="s">
-        <v>752</v>
-      </c>
-      <c r="DX30" t="s">
-        <v>4069</v>
-      </c>
-      <c r="DY30" t="s">
-        <v>3390</v>
-      </c>
-      <c r="DZ30" t="s">
-        <v>4792</v>
-      </c>
-      <c r="EA30" t="s">
-        <v>5205</v>
-      </c>
-      <c r="EB30" t="s">
-        <v>5206</v>
-      </c>
-      <c r="EC30" t="s">
-        <v>4330</v>
-      </c>
-      <c r="ED30" t="s">
-        <v>5207</v>
-      </c>
-      <c r="EE30" t="s">
-        <v>5208</v>
-      </c>
-      <c r="EF30" t="s">
-        <v>5209</v>
-      </c>
-      <c r="EG30" t="s">
-        <v>5210</v>
-      </c>
-      <c r="EH30" t="s">
-        <v>5211</v>
-      </c>
-      <c r="EI30" t="s">
-        <v>5212</v>
-      </c>
-      <c r="EJ30" t="s">
-        <v>5213</v>
-      </c>
-      <c r="EK30" t="s">
-        <v>5214</v>
-      </c>
-      <c r="EL30" t="s">
-        <v>5215</v>
-      </c>
-      <c r="EM30" t="s">
-        <v>4233</v>
-      </c>
-      <c r="EN30" t="s">
-        <v>5216</v>
-      </c>
-      <c r="EO30" t="s">
-        <v>5217</v>
-      </c>
-      <c r="EP30" t="s">
-        <v>5218</v>
-      </c>
-      <c r="EQ30" t="s">
-        <v>5219</v>
-      </c>
-      <c r="ER30" t="s">
-        <v>5220</v>
-      </c>
-      <c r="ES30" t="s">
-        <v>3840</v>
-      </c>
-      <c r="ET30" t="s">
-        <v>5221</v>
-      </c>
-      <c r="EU30" t="s">
-        <v>5222</v>
-      </c>
-      <c r="EV30" t="s">
-        <v>5223</v>
-      </c>
-      <c r="EW30" t="s">
-        <v>1662</v>
-      </c>
-      <c r="EX30" t="s">
-        <v>5167</v>
-      </c>
-      <c r="EY30" t="s">
-        <v>5224</v>
-      </c>
-      <c r="EZ30" t="s">
-        <v>5225</v>
-      </c>
-      <c r="FA30" t="s">
-        <v>5226</v>
-      </c>
-      <c r="FB30" t="s">
-        <v>5227</v>
-      </c>
-      <c r="FC30" t="s">
-        <v>3137</v>
-      </c>
-      <c r="FD30" t="s">
-        <v>5228</v>
-      </c>
-      <c r="FE30" t="s">
-        <v>5229</v>
-      </c>
-      <c r="FF30" t="s">
-        <v>5230</v>
-      </c>
-      <c r="FG30" t="s">
-        <v>3335</v>
-      </c>
-      <c r="FH30" t="s">
-        <v>5231</v>
-      </c>
-      <c r="FI30" t="s">
-        <v>5232</v>
-      </c>
-      <c r="FJ30" t="s">
-        <v>5233</v>
-      </c>
-      <c r="FK30" t="s">
-        <v>5234</v>
-      </c>
-      <c r="FL30" t="s">
-        <v>5235</v>
-      </c>
-      <c r="FM30" t="s">
-        <v>5236</v>
-      </c>
-      <c r="FN30" t="s">
-        <v>5237</v>
-      </c>
-      <c r="FO30" t="s">
-        <v>5238</v>
-      </c>
-      <c r="FP30" t="s">
-        <v>5239</v>
-      </c>
-      <c r="FQ30" t="s">
-        <v>5240</v>
-      </c>
-      <c r="FR30" t="s">
-        <v>1814</v>
-      </c>
-      <c r="FS30" t="s">
-        <v>5241</v>
-      </c>
-      <c r="FT30" t="s">
-        <v>5242</v>
-      </c>
-      <c r="FU30" t="s">
-        <v>5243</v>
-      </c>
-      <c r="FV30" t="s">
-        <v>5160</v>
-      </c>
-      <c r="FW30" t="s">
-        <v>1605</v>
-      </c>
-      <c r="FX30" t="s">
-        <v>5244</v>
-      </c>
-      <c r="FY30" t="s">
-        <v>5245</v>
-      </c>
-      <c r="FZ30" t="s">
-        <v>5246</v>
-      </c>
-      <c r="GA30" t="s">
-        <v>5247</v>
-      </c>
-      <c r="GB30" t="s">
-        <v>5248</v>
-      </c>
-      <c r="GC30" t="s">
-        <v>5092</v>
-      </c>
-      <c r="GD30" t="s">
-        <v>5249</v>
-      </c>
-      <c r="GE30" t="s">
-        <v>5250</v>
-      </c>
-      <c r="GF30" t="s">
-        <v>5251</v>
-      </c>
-      <c r="GG30" t="s">
-        <v>5252</v>
-      </c>
-      <c r="GH30" t="s">
-        <v>5253</v>
-      </c>
-      <c r="GI30" t="s">
-        <v>3987</v>
-      </c>
-      <c r="GJ30" t="s">
-        <v>3359</v>
-      </c>
-      <c r="GK30" t="s">
-        <v>5254</v>
-      </c>
-      <c r="GL30" t="s">
-        <v>5255</v>
-      </c>
-      <c r="GM30" t="s">
-        <v>5256</v>
-      </c>
-      <c r="GN30" t="s">
-        <v>5257</v>
-      </c>
-      <c r="GO30" t="s">
-        <v>5258</v>
-      </c>
-      <c r="GP30" t="s">
-        <v>5259</v>
-      </c>
-      <c r="GQ30" t="s">
-        <v>3376</v>
-      </c>
-      <c r="GR30" t="s">
-        <v>5260</v>
-      </c>
-      <c r="GS30" t="s">
-        <v>5261</v>
-      </c>
-      <c r="GT30" t="s">
-        <v>5262</v>
-      </c>
-      <c r="GU30" t="s">
-        <v>5263</v>
-      </c>
-      <c r="GV30" t="s">
-        <v>2622</v>
-      </c>
-      <c r="GW30" t="s">
-        <v>4759</v>
-      </c>
-      <c r="GX30" t="s">
-        <v>3070</v>
-      </c>
-      <c r="GY30" t="s">
-        <v>5264</v>
-      </c>
-      <c r="GZ30" t="s">
-        <v>5265</v>
-      </c>
-      <c r="HA30" t="s">
-        <v>5266</v>
-      </c>
-      <c r="HB30" t="s">
-        <v>5267</v>
-      </c>
-      <c r="HC30" t="s">
-        <v>1132</v>
-      </c>
-      <c r="HD30" t="s">
-        <v>5268</v>
-      </c>
-      <c r="HE30" t="s">
-        <v>2417</v>
-      </c>
-      <c r="HF30" t="s">
-        <v>5269</v>
-      </c>
-      <c r="HG30" t="s">
-        <v>5270</v>
-      </c>
-      <c r="HH30" t="s">
-        <v>5271</v>
-      </c>
-      <c r="HI30" t="s">
-        <v>5272</v>
-      </c>
-      <c r="HJ30" t="s">
-        <v>1247</v>
-      </c>
-      <c r="HK30" t="s">
-        <v>5273</v>
-      </c>
-      <c r="HL30" t="s">
-        <v>5274</v>
-      </c>
-      <c r="HM30" t="s">
-        <v>5275</v>
-      </c>
-      <c r="HN30" t="s">
-        <v>5276</v>
-      </c>
-      <c r="HO30" t="s">
-        <v>5277</v>
-      </c>
-      <c r="HP30" t="s">
-        <v>1946</v>
-      </c>
-      <c r="HQ30" t="s">
-        <v>3302</v>
-      </c>
-      <c r="HR30" t="s">
-        <v>5278</v>
-      </c>
-      <c r="HS30" t="s">
-        <v>5279</v>
-      </c>
-      <c r="HT30" t="s">
-        <v>5280</v>
-      </c>
-      <c r="HU30" t="s">
-        <v>5281</v>
-      </c>
-      <c r="HV30" t="s">
-        <v>5282</v>
-      </c>
-      <c r="HW30" t="s">
-        <v>5283</v>
-      </c>
-      <c r="HX30" t="s">
-        <v>5284</v>
-      </c>
-      <c r="HY30" t="s">
-        <v>5285</v>
-      </c>
-      <c r="HZ30" t="s">
-        <v>5286</v>
-      </c>
-      <c r="IA30" t="s">
-        <v>2821</v>
-      </c>
-      <c r="IB30" t="s">
-        <v>5287</v>
-      </c>
-      <c r="IC30" t="s">
-        <v>5288</v>
-      </c>
-      <c r="ID30" t="s">
-        <v>2049</v>
-      </c>
-      <c r="IE30" t="s">
-        <v>3751</v>
-      </c>
-      <c r="IF30" t="s">
-        <v>5289</v>
-      </c>
-      <c r="IG30" t="s">
-        <v>5290</v>
-      </c>
-      <c r="IH30" t="s">
-        <v>5291</v>
-      </c>
-      <c r="II30" t="s">
-        <v>5292</v>
-      </c>
-      <c r="IJ30" t="s">
-        <v>5293</v>
-      </c>
-      <c r="IK30" t="s">
-        <v>4529</v>
-      </c>
-      <c r="IL30" t="s">
-        <v>5294</v>
-      </c>
-      <c r="IM30" t="s">
-        <v>5295</v>
-      </c>
-      <c r="IN30" t="s">
-        <v>4712</v>
-      </c>
-      <c r="IO30" t="s">
-        <v>5206</v>
-      </c>
-      <c r="IP30" t="s">
-        <v>5296</v>
-      </c>
-      <c r="IQ30" t="s">
-        <v>5297</v>
-      </c>
-      <c r="IR30" t="s">
-        <v>5298</v>
-      </c>
-      <c r="IS30" t="s">
-        <v>2842</v>
-      </c>
-      <c r="IT30" t="s">
-        <v>5299</v>
-      </c>
-      <c r="IU30" t="s">
-        <v>5300</v>
-      </c>
-      <c r="IV30" t="s">
-        <v>2395</v>
-      </c>
-      <c r="IW30" t="s">
-        <v>2618</v>
-      </c>
-      <c r="IX30" t="s">
-        <v>5301</v>
-      </c>
-      <c r="IY30" t="s">
-        <v>867</v>
-      </c>
-      <c r="IZ30" t="s">
-        <v>5302</v>
-      </c>
-      <c r="JA30" t="s">
-        <v>5303</v>
-      </c>
-      <c r="JB30" t="s">
-        <v>5304</v>
-      </c>
-      <c r="JC30" t="s">
-        <v>5305</v>
-      </c>
-      <c r="JD30" t="s">
-        <v>5306</v>
-      </c>
-      <c r="JE30" t="s">
-        <v>5307</v>
-      </c>
-      <c r="JF30" t="s">
-        <v>5308</v>
-      </c>
-      <c r="JG30" t="s">
-        <v>924</v>
-      </c>
-      <c r="JH30" t="s">
-        <v>5309</v>
-      </c>
-      <c r="JI30" t="s">
-        <v>5310</v>
-      </c>
-      <c r="JJ30" t="s">
-        <v>5311</v>
-      </c>
-      <c r="JK30" t="s">
-        <v>5312</v>
-      </c>
-      <c r="JL30" t="s">
-        <v>2414</v>
-      </c>
-      <c r="JM30" t="s">
-        <v>5313</v>
-      </c>
-      <c r="JN30" t="s">
-        <v>5314</v>
-      </c>
-      <c r="JO30" t="s">
-        <v>5315</v>
-      </c>
-      <c r="JP30" t="s">
-        <v>5316</v>
-      </c>
-      <c r="JQ30" t="s">
-        <v>5317</v>
-      </c>
-      <c r="JR30" t="s">
-        <v>3513</v>
-      </c>
-      <c r="JS30" t="s">
-        <v>5318</v>
-      </c>
-      <c r="JT30" t="s">
-        <v>5319</v>
-      </c>
-      <c r="JU30" t="s">
-        <v>5320</v>
-      </c>
-      <c r="JV30" t="s">
-        <v>5321</v>
-      </c>
-      <c r="JW30" t="s">
-        <v>5322</v>
-      </c>
-      <c r="JX30" t="s">
-        <v>5323</v>
-      </c>
-      <c r="JY30" t="s">
-        <v>5324</v>
-      </c>
-      <c r="JZ30" t="s">
-        <v>5325</v>
-      </c>
-      <c r="KA30" t="s">
-        <v>4198</v>
-      </c>
-      <c r="KB30" t="s">
-        <v>5326</v>
-      </c>
-      <c r="KC30" t="s">
-        <v>5221</v>
-      </c>
-      <c r="KD30" t="s">
-        <v>5327</v>
-      </c>
-      <c r="KE30" t="s">
-        <v>5124</v>
-      </c>
-      <c r="KF30" t="s">
-        <v>5328</v>
-      </c>
-      <c r="KG30" t="s">
-        <v>4215</v>
-      </c>
-      <c r="KH30" t="s">
-        <v>5329</v>
-      </c>
-      <c r="KI30" t="s">
-        <v>5330</v>
-      </c>
-      <c r="KJ30" t="s">
-        <v>5331</v>
-      </c>
-      <c r="KK30" t="s">
-        <v>3557</v>
-      </c>
-      <c r="KL30" t="s">
-        <v>5332</v>
-      </c>
-      <c r="KM30" t="s">
-        <v>5333</v>
-      </c>
-      <c r="KN30" t="s">
-        <v>4503</v>
-      </c>
-      <c r="KO30" t="s">
-        <v>3729</v>
-      </c>
-      <c r="KP30" t="s">
-        <v>5334</v>
-      </c>
-      <c r="KQ30" t="s">
-        <v>5335</v>
-      </c>
-      <c r="KR30" t="s">
-        <v>5336</v>
-      </c>
-      <c r="KS30" t="s">
-        <v>5337</v>
-      </c>
-      <c r="KT30" t="s">
-        <v>5338</v>
-      </c>
-      <c r="KU30" t="s">
-        <v>972</v>
-      </c>
-      <c r="KV30" t="s">
-        <v>5339</v>
-      </c>
-      <c r="KW30" t="s">
-        <v>5340</v>
-      </c>
-      <c r="KX30" t="s">
-        <v>5341</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>